<commit_message>
Update chip report site 2026-05-04
</commit_message>
<xml_diff>
--- a/outputs/chip-report/台股盤後籌碼_2026-04-30.xlsx
+++ b/outputs/chip-report/台股盤後籌碼_2026-04-30.xlsx
@@ -1220,7 +1220,7 @@
     </row>
     <row r="52">
       <c r="A52" s="6" t="n">
-        <v>-56618</v>
+        <v>764572</v>
       </c>
       <c r="B52" s="6" t="n"/>
       <c r="C52" s="6" t="n"/>
@@ -1249,7 +1249,7 @@
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>224,544 - 281,162(4/15結算日淨額)</t>
+          <t>1,570,928 - 806,356(4/15結算日 BC 原始金額)</t>
         </is>
       </c>
       <c r="B54" s="7" t="n"/>
@@ -1305,7 +1305,7 @@
     </row>
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="6" t="n">
-        <v>105218</v>
+        <v>290293</v>
       </c>
       <c r="B58" s="6" t="n"/>
       <c r="C58" s="6" t="n"/>
@@ -1334,7 +1334,7 @@
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>85,285 - -19,933(4/15結算日淨額)</t>
+          <t>416,325 - 126,032(4/15結算日 BP 原始金額)</t>
         </is>
       </c>
       <c r="B60" s="7" t="n"/>
@@ -1505,7 +1505,7 @@
       <c r="F72" s="6" t="n"/>
       <c r="G72" s="6" t="n"/>
       <c r="I72" s="6" t="n">
-        <v>-212963</v>
+        <v>670397</v>
       </c>
       <c r="J72" s="6" t="n"/>
       <c r="K72" s="6" t="n"/>
@@ -1538,7 +1538,7 @@
       <c r="G74" s="7" t="n"/>
       <c r="I74" s="7" t="inlineStr">
         <is>
-          <t>-180,763 - 32,200(4/15結算日淨額)</t>
+          <t>1,841,559 - 1,171,162(4/15結算日 BC 原始金額)</t>
         </is>
       </c>
       <c r="J74" s="7" t="n"/>
@@ -1590,7 +1590,7 @@
       <c r="F78" s="6" t="n"/>
       <c r="G78" s="6" t="n"/>
       <c r="I78" s="6" t="n">
-        <v>-186393</v>
+        <v>157588</v>
       </c>
       <c r="J78" s="6" t="n"/>
       <c r="K78" s="6" t="n"/>
@@ -1623,7 +1623,7 @@
       <c r="G80" s="7" t="n"/>
       <c r="I80" s="7" t="inlineStr">
         <is>
-          <t>-87,054 - 99,339(4/15結算日淨額)</t>
+          <t>423,407 - 265,819(4/15結算日 BP 原始金額)</t>
         </is>
       </c>
       <c r="J80" s="7" t="n"/>

</xml_diff>